<commit_message>
lots of changes are made
</commit_message>
<xml_diff>
--- a/db/data/office_trans.xlsx
+++ b/db/data/office_trans.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pradeep\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pradeep\Desktop\storemgmt\db\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{787797B9-AA48-404D-A326-6297F2D0C16E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B966C7AC-3C5B-41E3-9F91-9E018F5E61BF}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="office_item_transactions" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">office_item_transactions!$A$1:$D$205</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">office_item_transactions!$A$1:$E$205</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">office_item_transactions!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>1-13-2.2</t>
   </si>
@@ -51,21 +51,17 @@
   <si>
     <t>temp_item_id</t>
   </si>
+  <si>
+    <t>amount</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,9 +88,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -375,16 +370,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D205"/>
-  <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:E205"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="1"/>
-    <col min="2" max="2" width="14.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="9.28515625" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="1"/>
+    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -397,2044 +390,2865 @@
       <c r="D1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A2"/>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2">
         <v>3</v>
       </c>
-      <c r="D2"/>
-    </row>
-    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A3"/>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="D3"/>
-    </row>
-    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A4"/>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
-      <c r="D4"/>
-    </row>
-    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A5"/>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5">
         <v>4</v>
       </c>
       <c r="C5">
         <v>2</v>
       </c>
-      <c r="D5"/>
-    </row>
-    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A6"/>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>5</v>
       </c>
       <c r="C6">
         <v>2</v>
       </c>
-      <c r="D6"/>
-    </row>
-    <row r="7" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A7"/>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>6</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
-      <c r="D7"/>
-    </row>
-    <row r="8" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A8"/>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>7</v>
       </c>
       <c r="C8">
         <v>7</v>
       </c>
-      <c r="D8"/>
-    </row>
-    <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9"/>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>8</v>
       </c>
       <c r="C9">
         <v>10</v>
       </c>
-      <c r="D9"/>
-    </row>
-    <row r="10" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A10"/>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>9</v>
       </c>
       <c r="C10">
         <v>2</v>
       </c>
-      <c r="D10"/>
-    </row>
-    <row r="11" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A11"/>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>10</v>
       </c>
       <c r="C11">
         <v>5</v>
       </c>
-      <c r="D11"/>
-    </row>
-    <row r="12" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12"/>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>11</v>
       </c>
       <c r="C12">
         <v>3</v>
       </c>
-      <c r="D12"/>
-    </row>
-    <row r="13" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A13"/>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B13">
         <v>12</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
-      <c r="D13"/>
-    </row>
-    <row r="14" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A14"/>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B14">
         <v>13</v>
       </c>
       <c r="C14">
         <v>2</v>
       </c>
-      <c r="D14"/>
-    </row>
-    <row r="15" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15"/>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B15">
         <v>14</v>
       </c>
       <c r="C15">
         <v>2</v>
       </c>
-      <c r="D15"/>
-    </row>
-    <row r="16" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A16"/>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B16">
         <v>15</v>
       </c>
       <c r="C16">
         <v>2</v>
       </c>
-      <c r="D16"/>
-    </row>
-    <row r="17" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A17"/>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17">
         <v>16</v>
       </c>
       <c r="C17">
         <v>2</v>
       </c>
-      <c r="D17"/>
-    </row>
-    <row r="18" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A18"/>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18">
         <v>17</v>
       </c>
       <c r="C18">
         <v>1</v>
       </c>
-      <c r="D18"/>
-    </row>
-    <row r="19" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A19"/>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19">
         <v>18</v>
       </c>
       <c r="C19">
         <v>2</v>
       </c>
-      <c r="D19"/>
-    </row>
-    <row r="20" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A20"/>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20">
         <v>19</v>
       </c>
       <c r="C20">
         <v>5</v>
       </c>
-      <c r="D20"/>
-    </row>
-    <row r="21" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A21"/>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21">
         <v>20</v>
       </c>
       <c r="C21">
         <v>2</v>
       </c>
-      <c r="D21"/>
-    </row>
-    <row r="22" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A22"/>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22">
         <v>21</v>
       </c>
       <c r="C22">
         <v>1</v>
       </c>
-      <c r="D22"/>
-    </row>
-    <row r="23" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A23"/>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23">
         <v>22</v>
       </c>
       <c r="C23">
         <v>4</v>
       </c>
-      <c r="D23"/>
-    </row>
-    <row r="24" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A24"/>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24">
         <v>23</v>
       </c>
       <c r="C24">
         <v>1</v>
       </c>
-      <c r="D24"/>
-    </row>
-    <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A25"/>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25">
         <v>24</v>
       </c>
       <c r="C25">
         <v>3</v>
       </c>
-      <c r="D25"/>
-    </row>
-    <row r="26" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A26"/>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B26">
         <v>25</v>
       </c>
       <c r="C26">
         <v>3</v>
       </c>
-      <c r="D26"/>
-    </row>
-    <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A27"/>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B27">
         <v>26</v>
       </c>
       <c r="C27">
         <v>14</v>
       </c>
-      <c r="D27"/>
-    </row>
-    <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A28"/>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B28">
         <v>27</v>
       </c>
       <c r="C28">
         <v>1</v>
       </c>
-      <c r="D28"/>
-    </row>
-    <row r="29" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A29"/>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B29">
         <v>28</v>
       </c>
       <c r="C29">
         <v>2</v>
       </c>
-      <c r="D29"/>
-    </row>
-    <row r="30" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A30"/>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B30">
         <v>29</v>
       </c>
       <c r="C30">
         <v>10</v>
       </c>
-      <c r="D30"/>
-    </row>
-    <row r="31" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A31"/>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B31">
         <v>30</v>
       </c>
       <c r="C31">
         <v>1</v>
       </c>
-      <c r="D31"/>
-    </row>
-    <row r="32" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A32"/>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B32">
         <v>31</v>
       </c>
       <c r="C32">
         <v>2</v>
       </c>
-      <c r="D32"/>
-    </row>
-    <row r="33" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A33"/>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B33">
         <v>32</v>
       </c>
       <c r="C33">
         <v>9</v>
       </c>
-      <c r="D33"/>
-    </row>
-    <row r="34" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A34"/>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B34">
         <v>33</v>
       </c>
       <c r="C34">
         <v>4</v>
       </c>
-      <c r="D34"/>
-    </row>
-    <row r="35" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A35"/>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B35">
         <v>34</v>
       </c>
       <c r="C35">
         <v>3</v>
       </c>
-      <c r="D35"/>
-    </row>
-    <row r="36" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A36"/>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B36">
         <v>35</v>
       </c>
       <c r="C36">
         <v>8</v>
       </c>
-      <c r="D36"/>
-    </row>
-    <row r="37" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A37"/>
+      <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B37">
         <v>36</v>
       </c>
       <c r="C37">
         <v>1</v>
       </c>
-      <c r="D37"/>
-    </row>
-    <row r="38" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A38"/>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B38">
         <v>37</v>
       </c>
       <c r="C38">
         <v>1</v>
       </c>
-      <c r="D38"/>
-    </row>
-    <row r="39" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A39"/>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B39">
         <v>38</v>
       </c>
       <c r="C39">
         <v>1</v>
       </c>
-      <c r="D39"/>
-    </row>
-    <row r="40" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A40"/>
+      <c r="D39">
+        <v>0</v>
+      </c>
+      <c r="E39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B40">
         <v>39</v>
       </c>
       <c r="C40">
         <v>1</v>
       </c>
-      <c r="D40"/>
-    </row>
-    <row r="41" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A41"/>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B41">
         <v>40</v>
       </c>
       <c r="C41">
         <v>1</v>
       </c>
-      <c r="D41"/>
-    </row>
-    <row r="42" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A42"/>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B42">
         <v>41</v>
       </c>
       <c r="C42">
         <v>1</v>
       </c>
-      <c r="D42"/>
-    </row>
-    <row r="43" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A43"/>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B43">
         <v>42</v>
       </c>
       <c r="C43">
         <v>1</v>
       </c>
-      <c r="D43"/>
-    </row>
-    <row r="44" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A44"/>
+      <c r="D43">
+        <v>0</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B44">
         <v>43</v>
       </c>
       <c r="C44">
         <v>1</v>
       </c>
-      <c r="D44"/>
-    </row>
-    <row r="45" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A45"/>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B45">
         <v>44</v>
       </c>
       <c r="C45">
         <v>1</v>
       </c>
-      <c r="D45"/>
-    </row>
-    <row r="46" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A46"/>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B46">
         <v>45</v>
       </c>
       <c r="C46">
         <v>3</v>
       </c>
-      <c r="D46"/>
-    </row>
-    <row r="47" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A47"/>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B47">
         <v>46</v>
       </c>
       <c r="C47">
         <v>3</v>
       </c>
-      <c r="D47"/>
-    </row>
-    <row r="48" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A48"/>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B48">
         <v>47</v>
       </c>
       <c r="C48">
         <v>2</v>
       </c>
-      <c r="D48"/>
-    </row>
-    <row r="49" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A49"/>
+      <c r="D48">
+        <v>0</v>
+      </c>
+      <c r="E48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B49">
         <v>48</v>
       </c>
       <c r="C49">
         <v>4</v>
       </c>
-      <c r="D49"/>
-    </row>
-    <row r="50" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A50"/>
+      <c r="D49">
+        <v>0</v>
+      </c>
+      <c r="E49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B50">
         <v>49</v>
       </c>
       <c r="C50">
         <v>4</v>
       </c>
-      <c r="D50"/>
-    </row>
-    <row r="51" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A51"/>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B51">
         <v>50</v>
       </c>
       <c r="C51">
         <v>21</v>
       </c>
-      <c r="D51"/>
-    </row>
-    <row r="52" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A52"/>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B52">
         <v>51</v>
       </c>
       <c r="C52">
         <v>4</v>
       </c>
-      <c r="D52"/>
-    </row>
-    <row r="53" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A53"/>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B53">
         <v>52</v>
       </c>
       <c r="C53">
         <v>1</v>
       </c>
-      <c r="D53"/>
-    </row>
-    <row r="54" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A54"/>
+      <c r="D53">
+        <v>0</v>
+      </c>
+      <c r="E53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B54">
         <v>53</v>
       </c>
       <c r="C54">
         <v>2</v>
       </c>
-      <c r="D54"/>
-    </row>
-    <row r="55" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A55"/>
+      <c r="D54">
+        <v>0</v>
+      </c>
+      <c r="E54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B55">
         <v>54</v>
       </c>
       <c r="C55">
         <v>6</v>
       </c>
-      <c r="D55"/>
-    </row>
-    <row r="56" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A56"/>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B56">
         <v>55</v>
       </c>
       <c r="C56">
         <v>2</v>
       </c>
-      <c r="D56"/>
-    </row>
-    <row r="57" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A57"/>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B57">
         <v>56</v>
       </c>
       <c r="C57">
         <v>1</v>
       </c>
-      <c r="D57"/>
-    </row>
-    <row r="58" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A58"/>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B58">
         <v>57</v>
       </c>
       <c r="C58">
         <v>1</v>
       </c>
-      <c r="D58"/>
-    </row>
-    <row r="59" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A59"/>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B59">
         <v>58</v>
       </c>
       <c r="C59">
         <v>1</v>
       </c>
-      <c r="D59"/>
-    </row>
-    <row r="60" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A60"/>
+      <c r="D59">
+        <v>0</v>
+      </c>
+      <c r="E59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B60">
         <v>59</v>
       </c>
       <c r="C60">
         <v>6</v>
       </c>
-      <c r="D60"/>
-    </row>
-    <row r="61" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A61"/>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B61">
         <v>60</v>
       </c>
       <c r="C61">
         <v>1</v>
       </c>
-      <c r="D61"/>
-    </row>
-    <row r="62" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A62"/>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B62">
         <v>61</v>
       </c>
       <c r="C62">
         <v>1</v>
       </c>
-      <c r="D62"/>
-    </row>
-    <row r="63" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A63"/>
+      <c r="D62">
+        <v>0</v>
+      </c>
+      <c r="E62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B63">
         <v>62</v>
       </c>
       <c r="C63">
         <v>1</v>
       </c>
-      <c r="D63"/>
-    </row>
-    <row r="64" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A64"/>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B64">
         <v>63</v>
       </c>
       <c r="C64">
         <v>1</v>
       </c>
-      <c r="D64"/>
-    </row>
-    <row r="65" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A65"/>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65">
         <v>64</v>
       </c>
       <c r="C65">
         <v>1</v>
       </c>
-      <c r="D65"/>
-    </row>
-    <row r="66" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A66"/>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="E65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B66">
         <v>65</v>
       </c>
       <c r="C66">
         <v>1</v>
       </c>
-      <c r="D66"/>
-    </row>
-    <row r="67" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A67"/>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B67">
         <v>66</v>
       </c>
       <c r="C67">
         <v>2</v>
       </c>
-      <c r="D67"/>
-    </row>
-    <row r="68" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A68"/>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B68">
         <v>67</v>
       </c>
       <c r="C68">
         <v>3</v>
       </c>
-      <c r="D68"/>
-    </row>
-    <row r="69" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A69"/>
+      <c r="D68">
+        <v>0</v>
+      </c>
+      <c r="E68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B69">
         <v>68</v>
       </c>
       <c r="C69">
         <v>3</v>
       </c>
-      <c r="D69"/>
-    </row>
-    <row r="70" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A70"/>
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="E69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B70">
         <v>69</v>
       </c>
       <c r="C70">
         <v>1</v>
       </c>
-      <c r="D70"/>
-    </row>
-    <row r="71" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A71"/>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B71">
         <v>70</v>
       </c>
       <c r="C71">
         <v>6</v>
       </c>
-      <c r="D71"/>
-    </row>
-    <row r="72" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A72"/>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B72">
         <v>71</v>
       </c>
       <c r="C72">
         <v>2</v>
       </c>
-      <c r="D72"/>
-    </row>
-    <row r="73" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A73"/>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B73">
         <v>72</v>
       </c>
       <c r="C73">
         <v>1</v>
       </c>
-      <c r="D73"/>
-    </row>
-    <row r="74" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A74"/>
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B74">
         <v>73</v>
       </c>
       <c r="C74">
         <v>2</v>
       </c>
-      <c r="D74"/>
-    </row>
-    <row r="75" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A75"/>
+      <c r="D74">
+        <v>0</v>
+      </c>
+      <c r="E74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B75">
         <v>74</v>
       </c>
       <c r="C75">
         <v>1</v>
       </c>
-      <c r="D75"/>
-    </row>
-    <row r="76" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A76"/>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B76">
         <v>76</v>
       </c>
       <c r="C76">
         <v>8</v>
       </c>
-      <c r="D76"/>
-    </row>
-    <row r="77" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A77"/>
+      <c r="D76">
+        <v>0</v>
+      </c>
+      <c r="E76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B77">
         <v>77</v>
       </c>
       <c r="C77">
         <v>4</v>
       </c>
-      <c r="D77"/>
-    </row>
-    <row r="78" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A78"/>
+      <c r="D77">
+        <v>0</v>
+      </c>
+      <c r="E77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B78">
         <v>78</v>
       </c>
       <c r="C78">
         <v>7</v>
       </c>
-      <c r="D78"/>
-    </row>
-    <row r="79" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A79"/>
+      <c r="D78">
+        <v>0</v>
+      </c>
+      <c r="E78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B79">
         <v>79</v>
       </c>
       <c r="C79">
         <v>3</v>
       </c>
-      <c r="D79"/>
-    </row>
-    <row r="80" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A80"/>
+      <c r="D79">
+        <v>0</v>
+      </c>
+      <c r="E79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B80">
         <v>80</v>
       </c>
       <c r="C80">
         <v>1</v>
       </c>
-      <c r="D80"/>
-    </row>
-    <row r="81" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A81"/>
+      <c r="D80">
+        <v>0</v>
+      </c>
+      <c r="E80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B81">
         <v>83</v>
       </c>
       <c r="C81">
         <v>1</v>
       </c>
-      <c r="D81"/>
-    </row>
-    <row r="82" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A82"/>
+      <c r="D81">
+        <v>0</v>
+      </c>
+      <c r="E81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B82">
         <v>85</v>
       </c>
       <c r="C82">
         <v>2</v>
       </c>
-      <c r="D82"/>
-    </row>
-    <row r="83" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A83"/>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="E82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B83">
         <v>87</v>
       </c>
       <c r="C83">
         <v>1</v>
       </c>
-      <c r="D83"/>
-    </row>
-    <row r="84" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A84"/>
+      <c r="D83">
+        <v>0</v>
+      </c>
+      <c r="E83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B84">
         <v>88</v>
       </c>
       <c r="C84">
         <v>3</v>
       </c>
-      <c r="D84"/>
-    </row>
-    <row r="85" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A85"/>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B85">
         <v>91</v>
       </c>
       <c r="C85">
         <v>1</v>
       </c>
-      <c r="D85"/>
-    </row>
-    <row r="86" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A86"/>
+      <c r="D85">
+        <v>0</v>
+      </c>
+      <c r="E85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B86">
         <v>94</v>
       </c>
       <c r="C86">
         <v>5</v>
       </c>
-      <c r="D86"/>
-    </row>
-    <row r="87" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A87"/>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B87">
         <v>95</v>
       </c>
       <c r="C87">
         <v>2</v>
       </c>
-      <c r="D87"/>
-    </row>
-    <row r="88" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A88"/>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B88">
         <v>96</v>
       </c>
       <c r="C88">
         <v>5</v>
       </c>
-      <c r="D88"/>
-    </row>
-    <row r="89" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A89"/>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B89">
         <v>97</v>
       </c>
       <c r="C89">
         <v>1</v>
       </c>
-      <c r="D89"/>
-    </row>
-    <row r="90" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A90"/>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B90">
         <v>98</v>
       </c>
       <c r="C90">
         <v>1</v>
       </c>
-      <c r="D90"/>
-    </row>
-    <row r="91" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A91"/>
+      <c r="D90">
+        <v>0</v>
+      </c>
+      <c r="E90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B91">
         <v>99</v>
       </c>
       <c r="C91">
         <v>1</v>
       </c>
-      <c r="D91"/>
-    </row>
-    <row r="92" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A92"/>
+      <c r="D91">
+        <v>0</v>
+      </c>
+      <c r="E91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B92">
         <v>100</v>
       </c>
       <c r="C92">
         <v>1</v>
       </c>
-      <c r="D92"/>
-    </row>
-    <row r="93" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A93"/>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B93">
         <v>101</v>
       </c>
       <c r="C93">
         <v>1</v>
       </c>
-      <c r="D93"/>
-    </row>
-    <row r="94" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A94"/>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B94">
         <v>102</v>
       </c>
       <c r="C94">
         <v>1</v>
       </c>
-      <c r="D94"/>
-    </row>
-    <row r="95" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A95"/>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B95">
         <v>103</v>
       </c>
       <c r="C95">
         <v>2</v>
       </c>
-      <c r="D95"/>
-    </row>
-    <row r="96" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A96"/>
+      <c r="D95">
+        <v>0</v>
+      </c>
+      <c r="E95">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B96">
         <v>104</v>
       </c>
       <c r="C96">
         <v>3</v>
       </c>
-      <c r="D96"/>
-    </row>
-    <row r="97" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A97"/>
+      <c r="D96">
+        <v>0</v>
+      </c>
+      <c r="E96">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B97">
         <v>105</v>
       </c>
       <c r="C97">
         <v>1</v>
       </c>
-      <c r="D97"/>
-    </row>
-    <row r="98" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A98"/>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B98">
         <v>106</v>
       </c>
       <c r="C98">
         <v>2</v>
       </c>
-      <c r="D98"/>
-    </row>
-    <row r="99" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A99"/>
+      <c r="D98">
+        <v>0</v>
+      </c>
+      <c r="E98">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B99">
         <v>107</v>
       </c>
       <c r="C99">
         <v>4</v>
       </c>
-      <c r="D99"/>
-    </row>
-    <row r="100" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A100"/>
+      <c r="D99">
+        <v>0</v>
+      </c>
+      <c r="E99">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B100">
         <v>108</v>
       </c>
       <c r="C100">
         <v>1</v>
       </c>
-      <c r="D100"/>
-    </row>
-    <row r="101" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A101"/>
+      <c r="D100">
+        <v>0</v>
+      </c>
+      <c r="E100">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B101">
         <v>109</v>
       </c>
       <c r="C101">
         <v>3</v>
       </c>
-      <c r="D101"/>
-    </row>
-    <row r="102" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A102"/>
+      <c r="D101">
+        <v>0</v>
+      </c>
+      <c r="E101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B102">
         <v>110</v>
       </c>
       <c r="C102">
         <v>1</v>
       </c>
-      <c r="D102"/>
-    </row>
-    <row r="103" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A103"/>
+      <c r="D102">
+        <v>0</v>
+      </c>
+      <c r="E102">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B103">
         <v>111</v>
       </c>
       <c r="C103">
         <v>1</v>
       </c>
-      <c r="D103"/>
-    </row>
-    <row r="104" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A104"/>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B104">
         <v>112</v>
       </c>
       <c r="C104">
         <v>1</v>
       </c>
-      <c r="D104"/>
-    </row>
-    <row r="105" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A105"/>
+      <c r="D104">
+        <v>0</v>
+      </c>
+      <c r="E104">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B105">
         <v>113</v>
       </c>
       <c r="C105">
         <v>1</v>
       </c>
-      <c r="D105"/>
-    </row>
-    <row r="106" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A106"/>
+      <c r="D105">
+        <v>0</v>
+      </c>
+      <c r="E105">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B106">
         <v>114</v>
       </c>
       <c r="C106">
         <v>1</v>
       </c>
-      <c r="D106"/>
-    </row>
-    <row r="107" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A107"/>
+      <c r="D106">
+        <v>0</v>
+      </c>
+      <c r="E106">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B107">
         <v>115</v>
       </c>
       <c r="C107">
         <v>1</v>
       </c>
-      <c r="D107"/>
-    </row>
-    <row r="108" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A108"/>
+      <c r="D107">
+        <v>0</v>
+      </c>
+      <c r="E107">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B108">
         <v>116</v>
       </c>
       <c r="C108">
         <v>1</v>
       </c>
-      <c r="D108"/>
-    </row>
-    <row r="109" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A109"/>
+      <c r="D108">
+        <v>0</v>
+      </c>
+      <c r="E108">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B109">
         <v>117</v>
       </c>
       <c r="C109">
         <v>1</v>
       </c>
-      <c r="D109"/>
-    </row>
-    <row r="110" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A110"/>
+      <c r="D109">
+        <v>0</v>
+      </c>
+      <c r="E109">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B110">
         <v>118</v>
       </c>
       <c r="C110">
         <v>3</v>
       </c>
-      <c r="D110"/>
-    </row>
-    <row r="111" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A111"/>
+      <c r="D110">
+        <v>0</v>
+      </c>
+      <c r="E110">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B111">
         <v>119</v>
       </c>
       <c r="C111">
         <v>2</v>
       </c>
-      <c r="D111"/>
-    </row>
-    <row r="112" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A112"/>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B112">
         <v>120</v>
       </c>
       <c r="C112">
         <v>1</v>
       </c>
-      <c r="D112"/>
-    </row>
-    <row r="113" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A113"/>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B113">
         <v>121</v>
       </c>
       <c r="C113">
         <v>2</v>
       </c>
-      <c r="D113"/>
-    </row>
-    <row r="114" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A114"/>
+      <c r="D113">
+        <v>0</v>
+      </c>
+      <c r="E113">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B114">
         <v>122</v>
       </c>
       <c r="C114">
         <v>1</v>
       </c>
-      <c r="D114"/>
-    </row>
-    <row r="115" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A115"/>
+      <c r="D114">
+        <v>0</v>
+      </c>
+      <c r="E114">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B115">
         <v>123</v>
       </c>
       <c r="C115">
         <v>1</v>
       </c>
-      <c r="D115"/>
-    </row>
-    <row r="116" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A116"/>
+      <c r="D115">
+        <v>0</v>
+      </c>
+      <c r="E115">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B116">
         <v>124</v>
       </c>
       <c r="C116">
         <v>1</v>
       </c>
-      <c r="D116"/>
-    </row>
-    <row r="117" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A117"/>
+      <c r="D116">
+        <v>0</v>
+      </c>
+      <c r="E116">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B117">
         <v>125</v>
       </c>
       <c r="C117">
         <v>1</v>
       </c>
-      <c r="D117"/>
-    </row>
-    <row r="118" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A118"/>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B118">
         <v>126</v>
       </c>
       <c r="C118">
         <v>2</v>
       </c>
-      <c r="D118"/>
-    </row>
-    <row r="119" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A119"/>
+      <c r="D118">
+        <v>0</v>
+      </c>
+      <c r="E118">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B119">
         <v>127</v>
       </c>
       <c r="C119">
         <v>5</v>
       </c>
-      <c r="D119"/>
-    </row>
-    <row r="120" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A120"/>
+      <c r="D119">
+        <v>0</v>
+      </c>
+      <c r="E119">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B120">
         <v>128</v>
       </c>
       <c r="C120">
         <v>1</v>
       </c>
-      <c r="D120"/>
-    </row>
-    <row r="121" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A121"/>
+      <c r="D120">
+        <v>0</v>
+      </c>
+      <c r="E120">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B121">
         <v>129</v>
       </c>
       <c r="C121">
         <v>2</v>
       </c>
-      <c r="D121"/>
-    </row>
-    <row r="122" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A122"/>
+      <c r="D121">
+        <v>0</v>
+      </c>
+      <c r="E121">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B122">
         <v>130</v>
       </c>
       <c r="C122">
         <v>2</v>
       </c>
-      <c r="D122"/>
-    </row>
-    <row r="123" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A123"/>
+      <c r="D122">
+        <v>0</v>
+      </c>
+      <c r="E122">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B123">
         <v>131</v>
       </c>
       <c r="C123">
         <v>6</v>
       </c>
-      <c r="D123"/>
-    </row>
-    <row r="124" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A124"/>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B124">
         <v>132</v>
       </c>
       <c r="C124">
         <v>1</v>
       </c>
-      <c r="D124"/>
-    </row>
-    <row r="125" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A125"/>
+      <c r="D124">
+        <v>0</v>
+      </c>
+      <c r="E124">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B125">
         <v>133</v>
       </c>
       <c r="C125">
         <v>2</v>
       </c>
-      <c r="D125"/>
-    </row>
-    <row r="126" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A126"/>
+      <c r="D125">
+        <v>0</v>
+      </c>
+      <c r="E125">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B126">
         <v>134</v>
       </c>
       <c r="C126">
         <v>1</v>
       </c>
-      <c r="D126"/>
-    </row>
-    <row r="127" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A127"/>
+      <c r="D126">
+        <v>0</v>
+      </c>
+      <c r="E126">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B127">
         <v>135</v>
       </c>
       <c r="C127">
         <v>1</v>
       </c>
-      <c r="D127"/>
-    </row>
-    <row r="128" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A128"/>
+      <c r="D127">
+        <v>0</v>
+      </c>
+      <c r="E127">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B128">
         <v>136</v>
       </c>
       <c r="C128">
         <v>1</v>
       </c>
-      <c r="D128"/>
-    </row>
-    <row r="129" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A129"/>
+      <c r="D128">
+        <v>0</v>
+      </c>
+      <c r="E128">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B129">
         <v>137</v>
       </c>
       <c r="C129">
         <v>1</v>
       </c>
-      <c r="D129"/>
-    </row>
-    <row r="130" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A130"/>
+      <c r="D129">
+        <v>0</v>
+      </c>
+      <c r="E129">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B130">
         <v>138</v>
       </c>
       <c r="C130">
         <v>4</v>
       </c>
-      <c r="D130"/>
-    </row>
-    <row r="131" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A131"/>
+      <c r="D130">
+        <v>0</v>
+      </c>
+      <c r="E130">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B131">
         <v>139</v>
       </c>
       <c r="C131">
         <v>3</v>
       </c>
-      <c r="D131"/>
-    </row>
-    <row r="132" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A132"/>
+      <c r="D131">
+        <v>0</v>
+      </c>
+      <c r="E131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B132">
         <v>140</v>
       </c>
       <c r="C132">
         <v>1</v>
       </c>
-      <c r="D132"/>
-    </row>
-    <row r="133" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A133"/>
+      <c r="D132">
+        <v>0</v>
+      </c>
+      <c r="E132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B133">
         <v>141</v>
       </c>
       <c r="C133">
         <v>5</v>
       </c>
-      <c r="D133"/>
-    </row>
-    <row r="134" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A134"/>
+      <c r="D133">
+        <v>0</v>
+      </c>
+      <c r="E133">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B134">
         <v>142</v>
       </c>
       <c r="C134">
         <v>4</v>
       </c>
-      <c r="D134"/>
-    </row>
-    <row r="135" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A135"/>
+      <c r="D134">
+        <v>0</v>
+      </c>
+      <c r="E134">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B135">
         <v>143</v>
       </c>
       <c r="C135">
         <v>2</v>
       </c>
-      <c r="D135"/>
-    </row>
-    <row r="136" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A136"/>
+      <c r="D135">
+        <v>0</v>
+      </c>
+      <c r="E135">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B136">
         <v>144</v>
       </c>
       <c r="C136">
         <v>1</v>
       </c>
-      <c r="D136"/>
-    </row>
-    <row r="137" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A137"/>
+      <c r="D136">
+        <v>0</v>
+      </c>
+      <c r="E136">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B137">
         <v>145</v>
       </c>
       <c r="C137">
         <v>1</v>
       </c>
-      <c r="D137"/>
-    </row>
-    <row r="138" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A138"/>
+      <c r="D137">
+        <v>0</v>
+      </c>
+      <c r="E137">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B138">
         <v>146</v>
       </c>
       <c r="C138">
         <v>1</v>
       </c>
-      <c r="D138"/>
-    </row>
-    <row r="139" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A139"/>
+      <c r="D138">
+        <v>0</v>
+      </c>
+      <c r="E138">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B139">
         <v>147</v>
       </c>
       <c r="C139">
         <v>1</v>
       </c>
-      <c r="D139"/>
-    </row>
-    <row r="140" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A140"/>
+      <c r="D139">
+        <v>0</v>
+      </c>
+      <c r="E139">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B140">
         <v>148</v>
       </c>
-      <c r="C140"/>
-      <c r="D140"/>
-    </row>
-    <row r="141" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A141"/>
+      <c r="C140">
+        <v>1</v>
+      </c>
+      <c r="D140">
+        <v>0</v>
+      </c>
+      <c r="E140">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B141">
         <v>149</v>
       </c>
       <c r="C141">
         <v>5</v>
       </c>
-      <c r="D141"/>
-    </row>
-    <row r="142" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A142"/>
+      <c r="D141">
+        <v>0</v>
+      </c>
+      <c r="E141">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B142">
         <v>150</v>
       </c>
       <c r="C142">
         <v>3</v>
       </c>
-      <c r="D142"/>
-    </row>
-    <row r="143" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A143"/>
+      <c r="D142">
+        <v>0</v>
+      </c>
+      <c r="E142">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B143">
         <v>151</v>
       </c>
       <c r="C143">
         <v>6</v>
       </c>
-      <c r="D143"/>
-    </row>
-    <row r="144" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A144"/>
+      <c r="D143">
+        <v>0</v>
+      </c>
+      <c r="E143">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B144">
         <v>152</v>
       </c>
       <c r="C144">
         <v>2</v>
       </c>
-      <c r="D144"/>
-    </row>
-    <row r="145" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A145"/>
+      <c r="D144">
+        <v>0</v>
+      </c>
+      <c r="E144">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B145">
         <v>153</v>
       </c>
       <c r="C145">
         <v>4</v>
       </c>
-      <c r="D145"/>
-    </row>
-    <row r="146" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A146"/>
+      <c r="D145">
+        <v>0</v>
+      </c>
+      <c r="E145">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B146">
         <v>154</v>
       </c>
       <c r="C146">
         <v>1</v>
       </c>
-      <c r="D146"/>
-    </row>
-    <row r="147" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A147"/>
+      <c r="D146">
+        <v>0</v>
+      </c>
+      <c r="E146">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B147">
         <v>155</v>
       </c>
       <c r="C147">
         <v>1</v>
       </c>
-      <c r="D147"/>
-    </row>
-    <row r="148" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A148"/>
+      <c r="D147">
+        <v>0</v>
+      </c>
+      <c r="E147">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B148">
         <v>156</v>
       </c>
       <c r="C148">
         <v>1</v>
       </c>
-      <c r="D148"/>
-    </row>
-    <row r="149" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A149"/>
+      <c r="D148">
+        <v>0</v>
+      </c>
+      <c r="E148">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B149">
         <v>157</v>
       </c>
       <c r="C149" t="s">
         <v>0</v>
       </c>
-      <c r="D149"/>
-    </row>
-    <row r="150" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A150"/>
+      <c r="D149">
+        <v>0</v>
+      </c>
+      <c r="E149">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B150">
         <v>158</v>
       </c>
       <c r="C150">
         <v>1</v>
       </c>
-      <c r="D150"/>
-    </row>
-    <row r="151" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A151"/>
+      <c r="D150">
+        <v>0</v>
+      </c>
+      <c r="E150">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B151">
         <v>159</v>
       </c>
       <c r="C151">
         <v>1</v>
       </c>
-      <c r="D151"/>
-    </row>
-    <row r="152" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A152"/>
+      <c r="D151">
+        <v>0</v>
+      </c>
+      <c r="E151">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B152">
         <v>160</v>
       </c>
       <c r="C152">
         <v>1</v>
       </c>
-      <c r="D152"/>
-    </row>
-    <row r="153" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A153"/>
+      <c r="D152">
+        <v>0</v>
+      </c>
+      <c r="E152">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B153">
         <v>161</v>
       </c>
       <c r="C153">
         <v>8</v>
       </c>
-      <c r="D153"/>
-    </row>
-    <row r="154" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A154"/>
+      <c r="D153">
+        <v>0</v>
+      </c>
+      <c r="E153">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B154">
         <v>162</v>
       </c>
       <c r="C154">
         <v>1</v>
       </c>
-      <c r="D154"/>
-    </row>
-    <row r="155" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A155"/>
+      <c r="D154">
+        <v>0</v>
+      </c>
+      <c r="E154">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B155">
         <v>163</v>
       </c>
       <c r="C155">
         <v>1</v>
       </c>
-      <c r="D155"/>
-    </row>
-    <row r="156" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A156"/>
+      <c r="D155">
+        <v>0</v>
+      </c>
+      <c r="E155">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B156">
         <v>164</v>
       </c>
       <c r="C156">
         <v>1</v>
       </c>
-      <c r="D156"/>
-    </row>
-    <row r="157" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A157"/>
+      <c r="D156">
+        <v>0</v>
+      </c>
+      <c r="E156">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B157">
         <v>165</v>
       </c>
       <c r="C157">
         <v>1</v>
       </c>
-      <c r="D157"/>
-    </row>
-    <row r="158" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A158"/>
+      <c r="D157">
+        <v>0</v>
+      </c>
+      <c r="E157">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B158">
         <v>166</v>
       </c>
       <c r="C158">
         <v>2</v>
       </c>
-      <c r="D158"/>
-    </row>
-    <row r="159" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A159"/>
+      <c r="D158">
+        <v>0</v>
+      </c>
+      <c r="E158">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B159">
         <v>167</v>
       </c>
       <c r="C159">
         <v>1</v>
       </c>
-      <c r="D159"/>
-    </row>
-    <row r="160" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A160"/>
+      <c r="D159">
+        <v>0</v>
+      </c>
+      <c r="E159">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B160">
         <v>168</v>
       </c>
       <c r="C160">
         <v>1</v>
       </c>
-      <c r="D160"/>
-    </row>
-    <row r="161" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A161"/>
+      <c r="D160">
+        <v>0</v>
+      </c>
+      <c r="E160">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B161">
         <v>169</v>
       </c>
       <c r="C161">
         <v>12</v>
       </c>
-      <c r="D161"/>
-    </row>
-    <row r="162" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A162"/>
+      <c r="D161">
+        <v>0</v>
+      </c>
+      <c r="E161">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B162">
         <v>170</v>
       </c>
       <c r="C162">
         <v>2</v>
       </c>
-      <c r="D162"/>
-    </row>
-    <row r="163" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A163"/>
+      <c r="D162">
+        <v>0</v>
+      </c>
+      <c r="E162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B163">
         <v>171</v>
       </c>
       <c r="C163">
         <v>2</v>
       </c>
-      <c r="D163"/>
-    </row>
-    <row r="164" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A164"/>
+      <c r="D163">
+        <v>0</v>
+      </c>
+      <c r="E163">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B164">
         <v>172</v>
       </c>
       <c r="C164">
         <v>2</v>
       </c>
-      <c r="D164"/>
-    </row>
-    <row r="165" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A165"/>
+      <c r="D164">
+        <v>0</v>
+      </c>
+      <c r="E164">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B165">
         <v>173</v>
       </c>
       <c r="C165">
         <v>3</v>
       </c>
-      <c r="D165"/>
-    </row>
-    <row r="166" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A166"/>
+      <c r="D165">
+        <v>0</v>
+      </c>
+      <c r="E165">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B166">
         <v>174</v>
       </c>
       <c r="C166">
         <v>2</v>
       </c>
-      <c r="D166"/>
-    </row>
-    <row r="167" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A167"/>
+      <c r="D166">
+        <v>0</v>
+      </c>
+      <c r="E166">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B167">
         <v>175</v>
       </c>
       <c r="C167">
         <v>23</v>
       </c>
-      <c r="D167"/>
-    </row>
-    <row r="168" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A168"/>
+      <c r="D167">
+        <v>0</v>
+      </c>
+      <c r="E167">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B168">
         <v>176</v>
       </c>
       <c r="C168">
         <v>1</v>
       </c>
-      <c r="D168"/>
-    </row>
-    <row r="169" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A169"/>
+      <c r="D168">
+        <v>0</v>
+      </c>
+      <c r="E168">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B169">
         <v>177</v>
       </c>
       <c r="C169">
         <v>1</v>
       </c>
-      <c r="D169"/>
-    </row>
-    <row r="170" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A170"/>
+      <c r="D169">
+        <v>0</v>
+      </c>
+      <c r="E169">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B170">
         <v>178</v>
       </c>
       <c r="C170">
         <v>2</v>
       </c>
-      <c r="D170"/>
-    </row>
-    <row r="171" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A171"/>
+      <c r="D170">
+        <v>0</v>
+      </c>
+      <c r="E170">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B171">
         <v>179</v>
       </c>
       <c r="C171">
         <v>1</v>
       </c>
-      <c r="D171"/>
-    </row>
-    <row r="172" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A172"/>
+      <c r="D171">
+        <v>0</v>
+      </c>
+      <c r="E171">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B172">
         <v>180</v>
       </c>
       <c r="C172">
         <v>6</v>
       </c>
-      <c r="D172"/>
-    </row>
-    <row r="173" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A173"/>
+      <c r="D172">
+        <v>0</v>
+      </c>
+      <c r="E172">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B173">
         <v>181</v>
       </c>
       <c r="C173">
         <v>1</v>
       </c>
-      <c r="D173"/>
-    </row>
-    <row r="174" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A174"/>
+      <c r="D173">
+        <v>0</v>
+      </c>
+      <c r="E173">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B174">
         <v>182</v>
       </c>
       <c r="C174">
         <v>1</v>
       </c>
-      <c r="D174"/>
-    </row>
-    <row r="175" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A175"/>
+      <c r="D174">
+        <v>0</v>
+      </c>
+      <c r="E174">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B175">
         <v>183</v>
       </c>
       <c r="C175">
         <v>6</v>
       </c>
-      <c r="D175"/>
-    </row>
-    <row r="176" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A176"/>
+      <c r="D175">
+        <v>0</v>
+      </c>
+      <c r="E175">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B176">
         <v>184</v>
       </c>
       <c r="C176">
         <v>1</v>
       </c>
-      <c r="D176"/>
-    </row>
-    <row r="177" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A177"/>
+      <c r="D176">
+        <v>0</v>
+      </c>
+      <c r="E176">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B177">
         <v>185</v>
       </c>
       <c r="C177">
         <v>2</v>
       </c>
-      <c r="D177"/>
-    </row>
-    <row r="178" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A178"/>
+      <c r="D177">
+        <v>0</v>
+      </c>
+      <c r="E177">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B178">
         <v>186</v>
       </c>
       <c r="C178">
         <v>4</v>
       </c>
-      <c r="D178"/>
-    </row>
-    <row r="179" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A179"/>
+      <c r="D178">
+        <v>0</v>
+      </c>
+      <c r="E178">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="179" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B179">
         <v>187</v>
       </c>
       <c r="C179">
         <v>3</v>
       </c>
-      <c r="D179"/>
-    </row>
-    <row r="180" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A180"/>
+      <c r="D179">
+        <v>0</v>
+      </c>
+      <c r="E179">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B180">
         <v>188</v>
       </c>
       <c r="C180">
         <v>1</v>
       </c>
-      <c r="D180"/>
-    </row>
-    <row r="181" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A181"/>
+      <c r="D180">
+        <v>0</v>
+      </c>
+      <c r="E180">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B181">
         <v>189</v>
       </c>
       <c r="C181">
         <v>3</v>
       </c>
-      <c r="D181"/>
-    </row>
-    <row r="182" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A182"/>
+      <c r="D181">
+        <v>0</v>
+      </c>
+      <c r="E181">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B182">
         <v>190</v>
       </c>
       <c r="C182">
         <v>1</v>
       </c>
-      <c r="D182"/>
-    </row>
-    <row r="183" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A183"/>
+      <c r="D182">
+        <v>0</v>
+      </c>
+      <c r="E182">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B183">
         <v>191</v>
       </c>
       <c r="C183">
         <v>1</v>
       </c>
-      <c r="D183"/>
-    </row>
-    <row r="184" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A184"/>
+      <c r="D183">
+        <v>0</v>
+      </c>
+      <c r="E183">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B184">
         <v>192</v>
       </c>
       <c r="C184">
         <v>1</v>
       </c>
-      <c r="D184"/>
-    </row>
-    <row r="185" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A185"/>
+      <c r="D184">
+        <v>0</v>
+      </c>
+      <c r="E184">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B185">
         <v>193</v>
       </c>
       <c r="C185">
         <v>3</v>
       </c>
-      <c r="D185"/>
-    </row>
-    <row r="186" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A186"/>
+      <c r="D185">
+        <v>0</v>
+      </c>
+      <c r="E185">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B186">
         <v>194</v>
       </c>
       <c r="C186">
         <v>1</v>
       </c>
-      <c r="D186"/>
-    </row>
-    <row r="187" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A187"/>
+      <c r="D186">
+        <v>0</v>
+      </c>
+      <c r="E186">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B187">
         <v>195</v>
       </c>
       <c r="C187">
         <v>1</v>
       </c>
-      <c r="D187"/>
-    </row>
-    <row r="188" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A188"/>
+      <c r="D187">
+        <v>0</v>
+      </c>
+      <c r="E187">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B188">
         <v>196</v>
       </c>
       <c r="C188">
         <v>1</v>
       </c>
-      <c r="D188"/>
-    </row>
-    <row r="189" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A189"/>
+      <c r="D188">
+        <v>0</v>
+      </c>
+      <c r="E188">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B189">
         <v>197</v>
       </c>
       <c r="C189">
         <v>1</v>
       </c>
-      <c r="D189"/>
-    </row>
-    <row r="190" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A190"/>
+      <c r="D189">
+        <v>0</v>
+      </c>
+      <c r="E189">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B190">
         <v>198</v>
       </c>
       <c r="C190">
         <v>3</v>
       </c>
-      <c r="D190"/>
-    </row>
-    <row r="191" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A191"/>
+      <c r="D190">
+        <v>0</v>
+      </c>
+      <c r="E190">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B191">
         <v>199</v>
       </c>
       <c r="C191">
         <v>1</v>
       </c>
-      <c r="D191"/>
-    </row>
-    <row r="192" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A192"/>
+      <c r="D191">
+        <v>0</v>
+      </c>
+      <c r="E191">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B192">
         <v>200</v>
       </c>
       <c r="C192">
         <v>2</v>
       </c>
-      <c r="D192"/>
-    </row>
-    <row r="193" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A193"/>
+      <c r="D192">
+        <v>0</v>
+      </c>
+      <c r="E192">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B193">
         <v>203</v>
       </c>
       <c r="C193">
         <v>1</v>
       </c>
-      <c r="D193"/>
-    </row>
-    <row r="194" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A194"/>
+      <c r="D193">
+        <v>0</v>
+      </c>
+      <c r="E193">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B194">
         <v>204</v>
       </c>
       <c r="C194">
         <v>3</v>
       </c>
-      <c r="D194"/>
-    </row>
-    <row r="195" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A195"/>
+      <c r="D194">
+        <v>0</v>
+      </c>
+      <c r="E194">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B195">
         <v>205</v>
       </c>
       <c r="C195">
         <v>1</v>
       </c>
-      <c r="D195"/>
-    </row>
-    <row r="196" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A196"/>
+      <c r="D195">
+        <v>0</v>
+      </c>
+      <c r="E195">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B196">
         <v>206</v>
       </c>
       <c r="C196">
         <v>2</v>
       </c>
-      <c r="D196"/>
-    </row>
-    <row r="197" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A197"/>
+      <c r="D196">
+        <v>0</v>
+      </c>
+      <c r="E196">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B197">
         <v>207</v>
       </c>
       <c r="C197">
         <v>6</v>
       </c>
-      <c r="D197"/>
-    </row>
-    <row r="198" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A198"/>
+      <c r="D197">
+        <v>0</v>
+      </c>
+      <c r="E197">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B198">
         <v>209</v>
       </c>
       <c r="C198">
         <v>1</v>
       </c>
-      <c r="D198"/>
-    </row>
-    <row r="199" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A199"/>
+      <c r="D198">
+        <v>0</v>
+      </c>
+      <c r="E198">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B199">
         <v>210</v>
       </c>
       <c r="C199">
         <v>1</v>
       </c>
-      <c r="D199"/>
-    </row>
-    <row r="200" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A200"/>
+      <c r="D199">
+        <v>0</v>
+      </c>
+      <c r="E199">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B200">
         <v>211</v>
       </c>
       <c r="C200">
         <v>1</v>
       </c>
-      <c r="D200"/>
-    </row>
-    <row r="201" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A201"/>
+      <c r="D200">
+        <v>0</v>
+      </c>
+      <c r="E200">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B201">
         <v>212</v>
       </c>
       <c r="C201">
         <v>1</v>
       </c>
-      <c r="D201"/>
-    </row>
-    <row r="202" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A202"/>
+      <c r="D201">
+        <v>0</v>
+      </c>
+      <c r="E201">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B202">
         <v>213</v>
       </c>
       <c r="C202">
         <v>1</v>
       </c>
-      <c r="D202"/>
-    </row>
-    <row r="203" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A203"/>
+      <c r="D202">
+        <v>0</v>
+      </c>
+      <c r="E202">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B203">
         <v>214</v>
       </c>
       <c r="C203">
         <v>3</v>
       </c>
-      <c r="D203"/>
-    </row>
-    <row r="204" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A204"/>
+      <c r="D203">
+        <v>0</v>
+      </c>
+      <c r="E203">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="204" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B204">
         <v>215</v>
       </c>
       <c r="C204">
         <v>1</v>
       </c>
-      <c r="D204"/>
-    </row>
-    <row r="205" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A205"/>
+      <c r="D204">
+        <v>0</v>
+      </c>
+      <c r="E204">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="205" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B205">
         <v>216</v>
       </c>
       <c r="C205">
         <v>1</v>
       </c>
-      <c r="D205"/>
+      <c r="D205">
+        <v>0</v>
+      </c>
+      <c r="E205">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>

</xml_diff>